<commit_message>
Fixed Pago Pago coordinates and patients needing vax columns
</commit_message>
<xml_diff>
--- a/data/American_Samoa_GIS_Demographics.xlsx
+++ b/data/American_Samoa_GIS_Demographics.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ikp9\R\USAPI\American Samoa\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ikp9\R\USAPI\American Samoa\AS_Coverage_Planning_Mapping_Dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{23B102AC-D7A8-4C41-AF07-4FDC6D9EFC99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3686E851-8764-4812-B5DF-D078C239285A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1708,14 +1708,14 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6855,10 +6855,10 @@
         <v>106</v>
       </c>
       <c r="H69" s="6">
-        <v>-14.252446000000001</v>
+        <v>-14.2733671054814</v>
       </c>
       <c r="I69" s="6">
-        <v>-170.70102800000001</v>
+        <v>-170.70362712815299</v>
       </c>
       <c r="J69" s="5">
         <v>3000</v>
@@ -7092,7 +7092,7 @@
         <v>822846</v>
       </c>
       <c r="M72" s="7">
-        <f t="shared" ref="M72:M103" si="6">IF(L72=0,0,L72/2589988.110336)</f>
+        <f t="shared" ref="M72:M89" si="6">IF(L72=0,0,L72/2589988.110336)</f>
         <v>0.31770261674801736</v>
       </c>
       <c r="N72" s="7">
@@ -11600,10 +11600,10 @@
         <v>106</v>
       </c>
       <c r="F63" s="6">
-        <v>-14.252446000000001</v>
+        <v>-14.2733671054814</v>
       </c>
       <c r="G63" s="6">
-        <v>-170.70102800000001</v>
+        <v>-170.70362712815299</v>
       </c>
       <c r="H63" s="5">
         <v>3000</v>
@@ -11986,7 +11986,7 @@
         <v>14932463</v>
       </c>
       <c r="K70" s="7">
-        <f t="shared" ref="K70:K101" si="6">IF(J70=0,0,J70/2589988.110336)</f>
+        <f t="shared" ref="K70:K82" si="6">IF(J70=0,0,J70/2589988.110336)</f>
         <v>5.7654561966552063</v>
       </c>
       <c r="L70" s="7">
@@ -13780,13 +13780,13 @@
       <c r="E11" s="14"/>
     </row>
     <row r="12" spans="1:5" ht="25.95" customHeight="1">
-      <c r="A12" s="18" t="s">
+      <c r="A12" s="20" t="s">
         <v>468</v>
       </c>
-      <c r="B12" s="18"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
     </row>
     <row r="13" spans="1:5" ht="43.95" customHeight="1">
       <c r="A13" s="12" t="s">
@@ -13803,12 +13803,12 @@
       <c r="A14" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="18" t="s">
         <v>471</v>
       </c>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="18"/>
     </row>
     <row r="15" spans="1:5" ht="43.95" customHeight="1">
       <c r="A15" s="12" t="s">
@@ -13825,12 +13825,12 @@
       <c r="A16" s="13" t="s">
         <v>474</v>
       </c>
-      <c r="B16" s="20" t="s">
+      <c r="B16" s="18" t="s">
         <v>475</v>
       </c>
-      <c r="C16" s="20"/>
-      <c r="D16" s="20"/>
-      <c r="E16" s="20"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="18"/>
+      <c r="E16" s="18"/>
     </row>
     <row r="17" spans="1:5" ht="43.95" customHeight="1">
       <c r="A17" s="12" t="s">
@@ -13847,12 +13847,12 @@
       <c r="A18" s="13" t="s">
         <v>478</v>
       </c>
-      <c r="B18" s="20" t="s">
+      <c r="B18" s="18" t="s">
         <v>479</v>
       </c>
-      <c r="C18" s="20"/>
-      <c r="D18" s="20"/>
-      <c r="E18" s="20"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18"/>
     </row>
     <row r="19" spans="1:5" ht="43.95" customHeight="1">
       <c r="A19" s="12" t="s">
@@ -13869,12 +13869,12 @@
       <c r="A20" s="13" t="s">
         <v>482</v>
       </c>
-      <c r="B20" s="20" t="s">
+      <c r="B20" s="18" t="s">
         <v>483</v>
       </c>
-      <c r="C20" s="20"/>
-      <c r="D20" s="20"/>
-      <c r="E20" s="20"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="18"/>
+      <c r="E20" s="18"/>
     </row>
     <row r="21" spans="1:5" ht="43.95" customHeight="1">
       <c r="A21" s="12" t="s">
@@ -13889,6 +13889,11 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="B14:E14"/>
     <mergeCell ref="B20:E20"/>
     <mergeCell ref="B21:E21"/>
     <mergeCell ref="B15:E15"/>
@@ -13896,11 +13901,6 @@
     <mergeCell ref="B17:E17"/>
     <mergeCell ref="B18:E18"/>
     <mergeCell ref="B19:E19"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A12:E12"/>
-    <mergeCell ref="B13:E13"/>
-    <mergeCell ref="B14:E14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>